<commit_message>
Deploying to gh-pages from @ ProjectesRecerca/he-prototype@9722d9d1c84022db06ee687d543bae38d15e57b5 🚀
</commit_message>
<xml_diff>
--- a/expanded-prototype/GrantRadar_Calls.xlsx
+++ b/expanded-prototype/GrantRadar_Calls.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\U107172\Desktop\Scripts\AplicacionsWeb\GrantRadar\v2.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDFB2B42-5658-4DB9-A329-29758EB76E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA5CB9E5-9557-4EBF-A514-EFB3CBDE43D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{90DF3CB5-27D5-4B95-8CAA-F538885FE317}"/>
   </bookViews>
@@ -7931,13 +7931,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -8000,11 +8000,9 @@
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
+        <left/>
         <right style="thin">
           <color rgb="FF000000"/>
         </right>
@@ -8032,9 +8030,11 @@
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
-        <left/>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
         <right style="thin">
           <color rgb="FF000000"/>
         </right>
@@ -8147,8 +8147,8 @@
     <tableColumn id="3" xr3:uid="{B2334D27-08C0-4B98-8B97-78C3CA45D849}" name="Column3"/>
     <tableColumn id="4" xr3:uid="{FC7406C8-DA4E-44D0-967D-82C5819B62A0}" name="Column4"/>
     <tableColumn id="22" xr3:uid="{906972EB-7345-4223-A6EE-AAF9956EE18E}" name="Column17" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{2A6E360D-B55E-48A6-A663-C5D68D27B266}" name="Column9" dataDxfId="0"/>
-    <tableColumn id="21" xr3:uid="{6FC69267-7189-43A4-91DD-0F08BC97367E}" name="Column15" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{2A6E360D-B55E-48A6-A663-C5D68D27B266}" name="Column9" dataDxfId="1"/>
+    <tableColumn id="21" xr3:uid="{6FC69267-7189-43A4-91DD-0F08BC97367E}" name="Column15" dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{5778F9E5-575A-4BE7-88AD-9E47E29955DD}" name="Column5"/>
     <tableColumn id="6" xr3:uid="{5CF6AB91-26B5-4641-9BC0-28C426CE6FC4}" name="Column6"/>
     <tableColumn id="7" xr3:uid="{E978B5E8-E943-44B5-AC85-CB558489FBF2}" name="Column7"/>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ ProjectesRecerca/he-prototype@0000adefa210eb45db9ecedbb662b45e217c5d16 🚀
</commit_message>
<xml_diff>
--- a/expanded-prototype/GrantRadar_Calls.xlsx
+++ b/expanded-prototype/GrantRadar_Calls.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\U107172\Desktop\Scripts\AplicacionsWeb\GrantRadar\v2.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA5CB9E5-9557-4EBF-A514-EFB3CBDE43D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20041179-C86F-4178-B55A-EDF9A33001B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{90DF3CB5-27D5-4B95-8CAA-F538885FE317}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet name="BDConvocatories" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -8479,6 +8480,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6CB36DF-D45A-42BA-94D5-B5740A47E1E1}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8A3F507-EE44-4235-89E7-91B4DCF979B0}">
   <dimension ref="A1:P995"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>